<commit_message>
feat(sample): add NC sample and tag label across sample meta flow
</commit_message>
<xml_diff>
--- a/bioinformatics-analysis/resources/sample-meta.xlsx
+++ b/bioinformatics-analysis/resources/sample-meta.xlsx
@@ -1,120 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\private\bioinfo-view\bio2023\code\bioinfo-view-be\bioinformatics-analysis\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC22886-5F3C-45B3-A2EB-E2C0E2FCC6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="27096" windowHeight="16296" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="27096" windowHeight="16296" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
-      <x14:workbookPr defaultImageDpi="32767"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" concurrentCalc="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>采样日期（YYYY-MM-DD）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>送测日期（YYYY-MM-DD）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>采样部位</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>样本类型</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>肿瘤含量</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>肿瘤样本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>患者识别号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>采样管品牌</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>标本类型</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FFFF0000"/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="11"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="11"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -130,37 +73,97 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -460,63 +463,93 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" customWidth="1"/>
+    <col width="24.6640625" bestFit="1" customWidth="1" style="4" min="1" max="2"/>
+    <col width="11.5546875" customWidth="1" style="4" min="7" max="7"/>
+    <col width="11.77734375" customWidth="1" style="4" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>采样日期（YYYY-MM-DD）</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>送测日期（YYYY-MM-DD）</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>采样部位</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>样本类型</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>肿瘤含量</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>肿瘤样本</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>NC??</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Tag??</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>患者识别号</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>采样管品牌</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>标本类型</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation sqref="D1:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"FFPE蜡块,新鲜组织,血液,脑脊液,胸水,其他体液,骨髓"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Arial"&amp;10&amp;K000000 Internal</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Arial"&amp;10 &amp;K000000_x000d_# Internal</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{06530cf4-8573-4c29-a912-bbcdac835909}" enabled="1" method="Standard" siteId="{ecaa386b-c8df-4ce0-ad01-740cbdb5ba55}" contentBits="2" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
fix(sample): correct template headers for nc and tag
</commit_message>
<xml_diff>
--- a/bioinformatics-analysis/resources/sample-meta.xlsx
+++ b/bioinformatics-analysis/resources/sample-meta.xlsx
@@ -509,12 +509,12 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>NC??</t>
+          <t>NC样本</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Tag??</t>
+          <t>Tag标签</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">

</xml_diff>